<commit_message>
case study for one coordinate + lcoe data
</commit_message>
<xml_diff>
--- a/input_data/technology_costs.xlsx
+++ b/input_data/technology_costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\opt_design_ammonia\input_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\Opt_H2\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBEF441-D6E0-44D2-9552-45FFB580C836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1713F71-B50B-4905-9683-E2F9ADC677FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2925" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2928" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="costs" sheetId="2" r:id="rId1"/>
@@ -21,19 +21,42 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Tobias Schließ</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{50E2EC63-F654-483F-AC93-A23EB03DBFFB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tobias Schließ:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+changed from "ecoinvent_312_reference"</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -622,13 +645,13 @@
     <t>Ref.</t>
   </si>
   <si>
-    <t>ecoinvent_312_reference</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1000_2050_base</t>
-  </si>
-  <si>
     <t>39%/CAPEX HB from Tonelli et al., similar assumption of 40% was used in Smith &amp; Torrente-Murciano, however based on personal comms we assume 20%,</t>
+  </si>
+  <si>
+    <t>ecoinvent-3.12-cutoff_remind-SSP1-PkBudg650_2030_08_full</t>
+  </si>
+  <si>
+    <t>ecoinvent-3.12-cutoff_remind-SSP1-PkBudg650_2050_08_full</t>
   </si>
 </sst>
 </file>
@@ -638,7 +661,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -681,6 +704,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1073,7 +1115,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1116,9 +1157,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1395,79 +1439,79 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O220"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.3125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.47265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.68359375" customWidth="1"/>
-    <col min="4" max="4" width="14.89453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.68359375" customWidth="1"/>
-    <col min="6" max="6" width="14.89453125" style="18" customWidth="1"/>
-    <col min="7" max="7" width="24.734375" style="18" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="17" customWidth="1"/>
+    <col min="7" max="7" width="24.77734375" style="17" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
-    <col min="9" max="9" width="23.1015625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.1015625" customWidth="1"/>
-    <col min="11" max="11" width="14.89453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.20703125" customWidth="1"/>
-    <col min="13" max="13" width="28.20703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="28.3671875" customWidth="1"/>
-    <col min="15" max="15" width="32.68359375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="31.7890625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1015625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.41796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.1015625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.3125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.89453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.20703125" customWidth="1"/>
-    <col min="23" max="23" width="31.41796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="24.7890625" customWidth="1"/>
-    <col min="27" max="27" width="18.3125" customWidth="1"/>
-    <col min="28" max="28" width="27.20703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15.89453125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.89453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.109375" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.21875" customWidth="1"/>
+    <col min="13" max="13" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.33203125" customWidth="1"/>
+    <col min="15" max="15" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.21875" customWidth="1"/>
+    <col min="23" max="23" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="24.77734375" customWidth="1"/>
+    <col min="27" max="27" width="18.33203125" customWidth="1"/>
+    <col min="28" max="28" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="14.7" thickBot="1">
+    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="B1" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="C1" s="45" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="19">
+      <c r="E1" s="18">
         <v>0.86</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="G1" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="34">
+      <c r="I1" s="33">
         <v>2025</v>
       </c>
-      <c r="J1" s="34">
+      <c r="J1" s="33">
         <v>2050</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="14.7" thickBot="1">
+    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1478,17 +1522,17 @@
         <f>B2</f>
         <v>30</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="14" t="s">
         <v>117</v>
       </c>
       <c r="F2"/>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="23" t="s">
         <v>27</v>
       </c>
       <c r="I2" s="2">
@@ -1499,14 +1543,14 @@
         <f t="shared" ref="J2:J25" si="1">C2</f>
         <v>30</v>
       </c>
-      <c r="K2" s="40" t="s">
+      <c r="K2" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="15" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="L2" s="14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -1518,17 +1562,17 @@
         <f>ROUND(753*E1,-1)</f>
         <v>650</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="16" t="s">
         <v>118</v>
       </c>
       <c r="F3"/>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="H3" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I3" s="4">
@@ -1539,15 +1583,15 @@
         <f t="shared" si="1"/>
         <v>650</v>
       </c>
-      <c r="K3" s="41" t="s">
+      <c r="K3" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="16" t="s">
         <v>118</v>
       </c>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
@@ -1558,15 +1602,15 @@
         <f>B4</f>
         <v>0.02</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F4"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27" t="s">
+      <c r="G4" s="25"/>
+      <c r="H4" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I4" s="4">
@@ -1577,14 +1621,14 @@
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="14.7" thickBot="1">
+      <c r="L4" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
@@ -1594,15 +1638,15 @@
       <c r="C5" s="8">
         <v>35</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F5"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27" t="s">
+      <c r="G5" s="25"/>
+      <c r="H5" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I5" s="4">
@@ -1613,14 +1657,14 @@
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="K5" s="41" t="s">
+      <c r="K5" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L5" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="L5" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1632,17 +1676,17 @@
         <f>ROUND(1188*E1,-1)</f>
         <v>1020</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="16" t="s">
         <v>118</v>
       </c>
       <c r="F6"/>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="27" t="s">
+      <c r="H6" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I6" s="4">
@@ -1653,14 +1697,14 @@
         <f t="shared" si="1"/>
         <v>1020</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K6" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.6" customHeight="1">
+    <row r="7" spans="1:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
@@ -1671,15 +1715,15 @@
         <f>B7</f>
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F7"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27" t="s">
+      <c r="G7" s="25"/>
+      <c r="H7" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I7" s="4">
@@ -1690,15 +1734,15 @@
         <f t="shared" si="1"/>
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="K7" s="41" t="s">
+      <c r="K7" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="16" t="s">
         <v>117</v>
       </c>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="1:13" ht="14.7" thickBot="1">
+    <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -1708,15 +1752,15 @@
       <c r="C8" s="8">
         <v>27</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F8"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27" t="s">
+      <c r="G8" s="25"/>
+      <c r="H8" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I8" s="4">
@@ -1727,14 +1771,14 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="K8" s="41" t="s">
+      <c r="K8" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L8" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="L8" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
@@ -1746,17 +1790,17 @@
         <f>ROUND(452*E1,-1)</f>
         <v>390</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="16" t="s">
         <v>118</v>
       </c>
       <c r="F9"/>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="26" t="s">
         <v>50</v>
       </c>
       <c r="I9" s="4">
@@ -1767,14 +1811,14 @@
         <f t="shared" si="1"/>
         <v>390</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K9" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="L9" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
@@ -1785,15 +1829,15 @@
         <f>B10</f>
         <v>0.02</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F10"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="27" t="s">
+      <c r="G10" s="25"/>
+      <c r="H10" s="26" t="s">
         <v>63</v>
       </c>
       <c r="I10" s="4">
@@ -1804,14 +1848,14 @@
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="K10" s="41" t="s">
+      <c r="K10" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L10" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+      <c r="L10" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
@@ -1822,15 +1866,15 @@
         <f>B11</f>
         <v>13</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F11"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27" t="s">
+      <c r="G11" s="25"/>
+      <c r="H11" s="26" t="s">
         <v>51</v>
       </c>
       <c r="I11" s="4">
@@ -1841,15 +1885,15 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="K11" s="41" t="s">
+      <c r="K11" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L11" s="17" t="s">
+      <c r="L11" s="16" t="s">
         <v>117</v>
       </c>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>24</v>
       </c>
@@ -1860,15 +1904,15 @@
         <f>ROUND(B12*(1+(C9-B9)/B9),-1)</f>
         <v>70</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F12"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="27" t="s">
+      <c r="G12" s="25"/>
+      <c r="H12" s="26" t="s">
         <v>52</v>
       </c>
       <c r="I12" s="4">
@@ -1879,14 +1923,14 @@
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="K12" s="41" t="s">
+      <c r="K12" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="L12" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+      <c r="L12" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1897,15 +1941,15 @@
         <f t="shared" ref="C13:C21" si="2">B13</f>
         <v>0.02</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F13"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27" t="s">
+      <c r="G13" s="25"/>
+      <c r="H13" s="26" t="s">
         <v>64</v>
       </c>
       <c r="I13" s="4">
@@ -1916,14 +1960,14 @@
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="K13" s="41" t="s">
+      <c r="K13" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L13" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+      <c r="L13" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
@@ -1934,15 +1978,15 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F14"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="27" t="s">
+      <c r="G14" s="25"/>
+      <c r="H14" s="26" t="s">
         <v>53</v>
       </c>
       <c r="I14" s="4">
@@ -1953,14 +1997,14 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="K14" s="41" t="s">
+      <c r="K14" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L14" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+      <c r="L14" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>4</v>
       </c>
@@ -1971,15 +2015,15 @@
         <f t="shared" si="2"/>
         <v>0.93</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F15"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="27" t="s">
+      <c r="G15" s="25"/>
+      <c r="H15" s="26" t="s">
         <v>54</v>
       </c>
       <c r="I15" s="4">
@@ -1990,15 +2034,15 @@
         <f t="shared" si="1"/>
         <v>0.93</v>
       </c>
-      <c r="K15" s="41" t="s">
+      <c r="K15" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L15" s="17" t="s">
+      <c r="L15" s="16" t="s">
         <v>117</v>
       </c>
       <c r="M15" s="1"/>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
@@ -2009,15 +2053,15 @@
         <f t="shared" si="2"/>
         <v>3.4999999999999976E-2</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F16"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27" t="s">
+      <c r="G16" s="25"/>
+      <c r="H16" s="26" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="4">
@@ -2028,14 +2072,14 @@
         <f t="shared" si="1"/>
         <v>3.4999999999999976E-2</v>
       </c>
-      <c r="K16" s="41" t="s">
+      <c r="K16" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15">
+      <c r="L16" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
@@ -2046,15 +2090,15 @@
         <f t="shared" si="2"/>
         <v>0.96500000000000008</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F17"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27" t="s">
+      <c r="G17" s="25"/>
+      <c r="H17" s="26" t="s">
         <v>57</v>
       </c>
       <c r="I17" s="4">
@@ -2065,14 +2109,14 @@
         <f t="shared" si="1"/>
         <v>0.96500000000000008</v>
       </c>
-      <c r="K17" s="41" t="s">
+      <c r="K17" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L17" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15">
+      <c r="L17" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>5</v>
       </c>
@@ -2083,15 +2127,15 @@
         <f t="shared" si="2"/>
         <v>0.91</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F18"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27" t="s">
+      <c r="G18" s="25"/>
+      <c r="H18" s="26" t="s">
         <v>46</v>
       </c>
       <c r="I18" s="4">
@@ -2102,14 +2146,14 @@
         <f t="shared" si="1"/>
         <v>0.91</v>
       </c>
-      <c r="K18" s="41" t="s">
+      <c r="K18" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L18" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15">
+      <c r="L18" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>30</v>
       </c>
@@ -2120,15 +2164,15 @@
         <f t="shared" si="2"/>
         <v>0.95399999999999996</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F19"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27" t="s">
+      <c r="G19" s="25"/>
+      <c r="H19" s="26" t="s">
         <v>47</v>
       </c>
       <c r="I19" s="4">
@@ -2139,14 +2183,14 @@
         <f t="shared" si="1"/>
         <v>0.95399999999999996</v>
       </c>
-      <c r="K19" s="41" t="s">
+      <c r="K19" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L19" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15">
+      <c r="L19" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
@@ -2157,15 +2201,15 @@
         <f t="shared" si="2"/>
         <v>0.95399999999999996</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F20"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="27" t="s">
+      <c r="G20" s="25"/>
+      <c r="H20" s="26" t="s">
         <v>48</v>
       </c>
       <c r="I20" s="4">
@@ -2176,16 +2220,16 @@
         <f t="shared" si="1"/>
         <v>0.95399999999999996</v>
       </c>
-      <c r="K20" s="41" t="s">
+      <c r="K20" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L20" s="17" t="s">
+      <c r="L20" s="16" t="s">
         <v>117</v>
       </c>
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
     </row>
-    <row r="21" spans="1:15" ht="14.7" thickBot="1">
+    <row r="21" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>14</v>
       </c>
@@ -2196,15 +2240,15 @@
         <f t="shared" si="2"/>
         <v>5.4000000000000001E-4</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F21"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27" t="s">
+      <c r="G21" s="25"/>
+      <c r="H21" s="26" t="s">
         <v>49</v>
       </c>
       <c r="I21" s="4">
@@ -2215,14 +2259,14 @@
         <f t="shared" si="1"/>
         <v>5.4000000000000001E-4</v>
       </c>
-      <c r="K21" s="41" t="s">
+      <c r="K21" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L21" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15">
+      <c r="L21" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>26</v>
       </c>
@@ -2233,17 +2277,17 @@
       <c r="C22" s="5">
         <v>500</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="16" t="s">
         <v>38</v>
       </c>
       <c r="E22" t="s">
         <v>120</v>
       </c>
       <c r="F22"/>
-      <c r="G22" s="29" t="s">
+      <c r="G22" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I22" s="4">
@@ -2254,7 +2298,7 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="K22" s="41" t="s">
+      <c r="K22" s="40" t="s">
         <v>93</v>
       </c>
       <c r="L22" t="s">
@@ -2263,7 +2307,7 @@
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>19</v>
       </c>
@@ -2274,15 +2318,15 @@
         <f>B23</f>
         <v>0.02</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="16" t="s">
         <v>118</v>
       </c>
       <c r="F23"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="27" t="s">
+      <c r="G23" s="29"/>
+      <c r="H23" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I23" s="4">
@@ -2293,17 +2337,17 @@
         <f t="shared" si="1"/>
         <v>0.02</v>
       </c>
-      <c r="K23" s="41" t="s">
+      <c r="K23" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L23" s="17" t="s">
+      <c r="L23" s="16" t="s">
         <v>118</v>
       </c>
       <c r="M23" s="1"/>
       <c r="N23" s="10"/>
       <c r="O23" s="10"/>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>12</v>
       </c>
@@ -2313,15 +2357,15 @@
       <c r="C24" s="5">
         <v>10</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="16" t="s">
         <v>2</v>
       </c>
       <c r="E24" t="s">
         <v>117</v>
       </c>
       <c r="F24"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="27" t="s">
+      <c r="G24" s="29"/>
+      <c r="H24" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I24" s="4">
@@ -2332,7 +2376,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K24" s="41" t="s">
+      <c r="K24" s="40" t="s">
         <v>2</v>
       </c>
       <c r="L24" t="s">
@@ -2347,7 +2391,7 @@
         <v>47.142857142857146</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="14.7" thickBot="1">
+    <row r="25" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>7</v>
       </c>
@@ -2357,15 +2401,15 @@
       <c r="C25" s="5">
         <v>0.7</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="D25" s="15" t="s">
         <v>3</v>
       </c>
       <c r="E25" t="s">
         <v>117</v>
       </c>
       <c r="F25"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="27" t="s">
+      <c r="G25" s="29"/>
+      <c r="H25" s="26" t="s">
         <v>42</v>
       </c>
       <c r="I25" s="4">
@@ -2376,14 +2420,14 @@
         <f t="shared" si="1"/>
         <v>0.7</v>
       </c>
-      <c r="K25" s="41" t="s">
+      <c r="K25" s="40" t="s">
         <v>3</v>
       </c>
       <c r="L25" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="14.7" thickBot="1">
+    <row r="26" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>65</v>
       </c>
@@ -2394,14 +2438,14 @@
         <f>B26</f>
         <v>20</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="16" t="s">
         <v>2</v>
       </c>
       <c r="F26"/>
-      <c r="G26" s="26" t="s">
+      <c r="G26" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="H26" s="27" t="s">
+      <c r="H26" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I26" s="4">
@@ -2412,14 +2456,14 @@
         <f t="shared" ref="J26:J35" si="4">C27</f>
         <v>200</v>
       </c>
-      <c r="K26" s="41" t="s">
+      <c r="K26" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="L26" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15">
+      <c r="L26" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -2430,15 +2474,15 @@
         <f>B27</f>
         <v>200</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="14" t="s">
         <v>37</v>
       </c>
       <c r="E27" t="s">
         <v>117</v>
       </c>
       <c r="F27"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="27" t="s">
+      <c r="G27" s="25"/>
+      <c r="H27" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I27" s="4">
@@ -2449,14 +2493,14 @@
         <f t="shared" si="4"/>
         <v>0.02</v>
       </c>
-      <c r="K27" s="41" t="s">
+      <c r="K27" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L27" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15">
+      <c r="L27" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>20</v>
       </c>
@@ -2467,15 +2511,15 @@
         <f>B28</f>
         <v>0.02</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="16" t="s">
         <v>3</v>
       </c>
       <c r="E28" t="s">
         <v>117</v>
       </c>
       <c r="F28"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="27" t="s">
+      <c r="G28" s="25"/>
+      <c r="H28" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I28" s="4">
@@ -2486,15 +2530,15 @@
         <f t="shared" si="4"/>
         <v>50</v>
       </c>
-      <c r="K28" s="41" t="s">
+      <c r="K28" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L28" s="17" t="s">
+      <c r="L28" s="16" t="s">
         <v>122</v>
       </c>
       <c r="M28" s="1"/>
     </row>
-    <row r="29" spans="1:15" ht="14.7" thickBot="1">
+    <row r="29" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>13</v>
       </c>
@@ -2504,17 +2548,17 @@
       <c r="C29" s="5">
         <v>50</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="16" t="s">
         <v>2</v>
       </c>
       <c r="E29" t="s">
         <v>122</v>
       </c>
       <c r="F29"/>
-      <c r="G29" s="26" t="s">
+      <c r="G29" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="H29" s="27" t="s">
+      <c r="H29" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I29" s="4">
@@ -2525,13 +2569,13 @@
         <f t="shared" si="4"/>
         <v>25.799999999999997</v>
       </c>
-      <c r="K29" s="41" t="s">
+      <c r="K29" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="L29" s="17"/>
+      <c r="L29" s="16"/>
       <c r="M29" s="1"/>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>104</v>
       </c>
@@ -2543,17 +2587,17 @@
         <f>B30</f>
         <v>25.799999999999997</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E30" s="17" t="s">
+      <c r="E30" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F30">
         <v>860</v>
       </c>
-      <c r="G30" s="26"/>
-      <c r="H30" s="27" t="s">
+      <c r="G30" s="25"/>
+      <c r="H30" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I30" s="4">
@@ -2564,10 +2608,10 @@
         <f t="shared" si="4"/>
         <v>0.01</v>
       </c>
-      <c r="K30" s="41" t="s">
+      <c r="K30" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L30" s="17" t="s">
+      <c r="L30" s="16" t="s">
         <v>118</v>
       </c>
       <c r="N30">
@@ -2575,7 +2619,7 @@
         <v>3.3333333333333335</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>105</v>
       </c>
@@ -2586,15 +2630,15 @@
         <f>B31</f>
         <v>0.01</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="17" t="s">
+      <c r="E31" s="16" t="s">
         <v>118</v>
       </c>
       <c r="F31"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="27" t="s">
+      <c r="G31" s="25"/>
+      <c r="H31" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I31" s="4">
@@ -2605,14 +2649,14 @@
         <f t="shared" si="4"/>
         <v>25</v>
       </c>
-      <c r="K31" s="41" t="s">
+      <c r="K31" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L31" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15">
+      <c r="L31" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>106</v>
       </c>
@@ -2622,15 +2666,15 @@
       <c r="C32" s="5">
         <v>25</v>
       </c>
-      <c r="D32" s="17" t="s">
+      <c r="D32" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E32" s="17" t="s">
+      <c r="E32" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F32"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="27" t="s">
+      <c r="G32" s="25"/>
+      <c r="H32" s="26" t="s">
         <v>55</v>
       </c>
       <c r="I32" s="4">
@@ -2641,14 +2685,14 @@
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="K32" s="41" t="s">
+      <c r="K32" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="L32" s="17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" ht="14.7" thickBot="1">
+      <c r="L32" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>107</v>
       </c>
@@ -2659,17 +2703,17 @@
         <f>B33</f>
         <v>4</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="D33" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="E33" s="16" t="s">
         <v>117</v>
       </c>
       <c r="F33"/>
-      <c r="G33" s="26" t="s">
+      <c r="G33" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="H33" s="27" t="s">
+      <c r="H33" s="26" t="s">
         <v>40</v>
       </c>
       <c r="I33" s="4">
@@ -2680,30 +2724,30 @@
         <f t="shared" si="4"/>
         <v>4300</v>
       </c>
-      <c r="K33" s="41" t="s">
+      <c r="K33" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="L33" s="17"/>
-    </row>
-    <row r="34" spans="1:15">
+      <c r="L33" s="16"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="20">
         <f>B58</f>
         <v>8600</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="21">
         <f>ROUND(B34/2,-1)</f>
         <v>4300</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E34" s="17"/>
+      <c r="E34" s="16"/>
       <c r="F34"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="27" t="s">
+      <c r="G34" s="25"/>
+      <c r="H34" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I34" s="4">
@@ -2714,15 +2758,15 @@
         <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
-      <c r="K34" s="41" t="s">
+      <c r="K34" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L34" s="17"/>
+      <c r="L34" s="16"/>
       <c r="M34" s="1"/>
       <c r="N34" s="10"/>
       <c r="O34" s="10"/>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>67</v>
       </c>
@@ -2733,13 +2777,13 @@
         <f>B35</f>
         <v>0.03</v>
       </c>
-      <c r="D35" s="17" t="s">
+      <c r="D35" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E35" s="17"/>
+      <c r="E35" s="16"/>
       <c r="F35"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="27" t="s">
+      <c r="G35" s="25"/>
+      <c r="H35" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I35" s="4">
@@ -2750,12 +2794,12 @@
         <f t="shared" si="4"/>
         <v>30</v>
       </c>
-      <c r="K35" s="41" t="s">
+      <c r="K35" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="L35" s="17"/>
-    </row>
-    <row r="36" spans="1:15">
+      <c r="L35" s="16"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>68</v>
       </c>
@@ -2766,13 +2810,13 @@
         <f>B36</f>
         <v>30</v>
       </c>
-      <c r="D36" s="17" t="s">
+      <c r="D36" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E36" s="17"/>
+      <c r="E36" s="16"/>
       <c r="F36"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="27" t="s">
+      <c r="G36" s="38"/>
+      <c r="H36" s="26" t="s">
         <v>111</v>
       </c>
       <c r="I36" s="4">
@@ -2783,12 +2827,12 @@
         <f>C40</f>
         <v>0.2</v>
       </c>
-      <c r="K36" s="17" t="s">
+      <c r="K36" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="L36" s="17"/>
-    </row>
-    <row r="37" spans="1:15">
+      <c r="L36" s="16"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>69</v>
       </c>
@@ -2799,13 +2843,13 @@
         <f>B37</f>
         <v>2</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E37" s="17"/>
+      <c r="E37" s="16"/>
       <c r="F37"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="27" t="s">
+      <c r="G37" s="25"/>
+      <c r="H37" s="26" t="s">
         <v>112</v>
       </c>
       <c r="I37" s="4">
@@ -2816,14 +2860,14 @@
         <f>C42</f>
         <v>0.1764</v>
       </c>
-      <c r="K37" s="41" t="s">
+      <c r="K37" s="40" t="s">
         <v>96</v>
       </c>
-      <c r="L37" s="17" t="s">
+      <c r="L37" s="16" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="16.8">
+    <row r="38" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>70</v>
       </c>
@@ -2833,13 +2877,13 @@
       <c r="C38" s="5">
         <v>5</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E38" s="17"/>
+      <c r="E38" s="16"/>
       <c r="F38"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="27" t="s">
+      <c r="G38" s="25"/>
+      <c r="H38" s="26" t="s">
         <v>103</v>
       </c>
       <c r="I38" s="4">
@@ -2849,14 +2893,14 @@
       <c r="J38" s="5">
         <v>0.4</v>
       </c>
-      <c r="K38" s="41" t="s">
+      <c r="K38" s="40" t="s">
         <v>95</v>
       </c>
-      <c r="L38" s="17" t="s">
+      <c r="L38" s="16" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="14.7" thickBot="1">
+    <row r="39" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>71</v>
       </c>
@@ -2866,13 +2910,13 @@
       <c r="C39" s="5">
         <v>5</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E39" s="17"/>
+      <c r="E39" s="16"/>
       <c r="F39"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="32" t="s">
+      <c r="G39" s="30"/>
+      <c r="H39" s="31" t="s">
         <v>85</v>
       </c>
       <c r="I39" s="6">
@@ -2883,13 +2927,13 @@
         <f>C48</f>
         <v>0.82299999999999995</v>
       </c>
-      <c r="K39" s="42" t="s">
+      <c r="K39" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="L39" s="17"/>
+      <c r="L39" s="16"/>
       <c r="M39" s="1"/>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>72</v>
       </c>
@@ -2899,15 +2943,15 @@
       <c r="C40" s="5">
         <v>0.2</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="17"/>
+      <c r="E40" s="16"/>
       <c r="F40"/>
-      <c r="G40" s="23" t="s">
+      <c r="G40" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="H40" s="24" t="s">
+      <c r="H40" s="23" t="s">
         <v>40</v>
       </c>
       <c r="I40" s="2">
@@ -2918,12 +2962,12 @@
         <f t="shared" ref="J40:J43" si="5">C44</f>
         <v>860</v>
       </c>
-      <c r="K40" s="25" t="s">
+      <c r="K40" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="L40" s="17"/>
-    </row>
-    <row r="41" spans="1:15">
+      <c r="L40" s="16"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>79</v>
       </c>
@@ -2934,12 +2978,12 @@
         <f>B41</f>
         <v>1</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="16" t="s">
         <v>80</v>
       </c>
       <c r="F41"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="27" t="s">
+      <c r="G41" s="25"/>
+      <c r="H41" s="26" t="s">
         <v>41</v>
       </c>
       <c r="I41" s="4">
@@ -2950,14 +2994,14 @@
         <f t="shared" si="5"/>
         <v>0.02</v>
       </c>
-      <c r="K41" s="28" t="s">
+      <c r="K41" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="L41" s="17" t="s">
+      <c r="L41" s="16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>108</v>
       </c>
@@ -2969,15 +3013,15 @@
         <f>B42</f>
         <v>0.1764</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="16" t="s">
         <v>92</v>
       </c>
       <c r="E42" t="s">
         <v>121</v>
       </c>
       <c r="F42"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="27" t="s">
+      <c r="G42" s="25"/>
+      <c r="H42" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I42" s="4">
@@ -2988,14 +3032,14 @@
         <f t="shared" si="5"/>
         <v>25</v>
       </c>
-      <c r="K42" s="28" t="s">
+      <c r="K42" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="L42" s="17" t="s">
+      <c r="L42" s="16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="14.7" thickBot="1">
+    <row r="43" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>109</v>
       </c>
@@ -3005,15 +3049,15 @@
       <c r="C43" s="5">
         <v>0.4</v>
       </c>
-      <c r="D43" s="17" t="s">
+      <c r="D43" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="E43" s="17" t="s">
+      <c r="E43" s="16" t="s">
         <v>122</v>
       </c>
       <c r="F43"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="37" t="s">
+      <c r="G43" s="35"/>
+      <c r="H43" s="36" t="s">
         <v>84</v>
       </c>
       <c r="I43" s="6">
@@ -3024,14 +3068,14 @@
         <f t="shared" si="5"/>
         <v>0.56299999999999994</v>
       </c>
-      <c r="K43" s="38" t="s">
+      <c r="K43" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="L43" s="16" t="s">
+      <c r="L43" s="15" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="44" spans="1:15">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>73</v>
       </c>
@@ -3043,14 +3087,14 @@
         <f>ROUND(0.2*C34,-1)</f>
         <v>860</v>
       </c>
-      <c r="D44" s="15" t="s">
+      <c r="D44" s="14" t="s">
         <v>100</v>
       </c>
       <c r="E44" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>74</v>
       </c>
@@ -3060,14 +3104,14 @@
       <c r="C45">
         <v>0.02</v>
       </c>
-      <c r="D45" s="17" t="s">
+      <c r="D45" s="16" t="s">
         <v>3</v>
       </c>
       <c r="E45" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="14.7" thickBot="1">
+    <row r="46" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
         <v>75</v>
       </c>
@@ -3078,11 +3122,11 @@
         <f>B46</f>
         <v>25</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="15" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:15">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>78</v>
       </c>
@@ -3094,7 +3138,7 @@
         <f>B47</f>
         <v>0.56299999999999994</v>
       </c>
-      <c r="D47" s="15" t="s">
+      <c r="D47" s="14" t="s">
         <v>101</v>
       </c>
       <c r="E47" t="s">
@@ -3103,7 +3147,7 @@
       <c r="F47"/>
       <c r="G47"/>
     </row>
-    <row r="48" spans="1:15" ht="14.7" thickBot="1">
+    <row r="48" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
         <v>110</v>
       </c>
@@ -3123,26 +3167,26 @@
       <c r="F48"/>
       <c r="G48"/>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F49"/>
       <c r="G49" s="10"/>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="G50"/>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F51"/>
-      <c r="G51" s="13"/>
-      <c r="H51" s="13"/>
-    </row>
-    <row r="52" spans="1:8" ht="14.7" thickBot="1">
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+    </row>
+    <row r="52" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>81</v>
       </c>
-      <c r="B52" s="13"/>
-      <c r="F52" s="13"/>
-    </row>
-    <row r="53" spans="1:8">
+      <c r="B52" s="12"/>
+      <c r="F52" s="12"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <f>130.44 / 105.418</f>
         <v>1.2373598436699613</v>
@@ -3153,8 +3197,8 @@
       <c r="F53"/>
       <c r="G53"/>
     </row>
-    <row r="54" spans="1:8" ht="14.7" thickBot="1">
-      <c r="A54" s="20">
+    <row r="54" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="19">
         <v>4192</v>
       </c>
       <c r="B54" s="8" t="s">
@@ -3162,9 +3206,9 @@
       </c>
       <c r="F54"/>
       <c r="G54"/>
-      <c r="H54" s="14"/>
-    </row>
-    <row r="55" spans="1:8">
+      <c r="H54" s="13"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B55">
         <f>20*365</f>
         <v>7300</v>
@@ -3172,21 +3216,21 @@
       <c r="F55"/>
       <c r="G55"/>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B56">
         <v>4935</v>
       </c>
       <c r="F56"/>
       <c r="G56"/>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B57">
         <v>10000</v>
       </c>
       <c r="F57"/>
       <c r="G57"/>
     </row>
-    <row r="58" spans="1:8" ht="14.7" thickBot="1">
+    <row r="58" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58">
         <f>B57*E1</f>
         <v>8600</v>
@@ -3194,7 +3238,7 @@
       <c r="F58"/>
       <c r="G58"/>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>116</v>
       </c>
@@ -3204,7 +3248,7 @@
       <c r="F59"/>
       <c r="G59"/>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>113</v>
       </c>
@@ -3214,7 +3258,7 @@
       <c r="F60"/>
       <c r="G60"/>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>114</v>
       </c>
@@ -3225,7 +3269,7 @@
       <c r="F61"/>
       <c r="G61"/>
     </row>
-    <row r="62" spans="1:8" ht="14.7" thickBot="1">
+    <row r="62" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>115</v>
       </c>
@@ -3236,607 +3280,607 @@
       <c r="F62"/>
       <c r="G62"/>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F63"/>
       <c r="G63"/>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F64"/>
       <c r="G64"/>
     </row>
-    <row r="65" spans="6:7">
+    <row r="65" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F65"/>
       <c r="G65"/>
     </row>
-    <row r="66" spans="6:7">
+    <row r="66" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F66"/>
       <c r="G66"/>
     </row>
-    <row r="67" spans="6:7">
+    <row r="67" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F67"/>
       <c r="G67"/>
     </row>
-    <row r="68" spans="6:7">
+    <row r="68" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F68"/>
       <c r="G68"/>
     </row>
-    <row r="69" spans="6:7">
+    <row r="69" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F69"/>
       <c r="G69"/>
     </row>
-    <row r="70" spans="6:7">
+    <row r="70" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F70"/>
       <c r="G70"/>
     </row>
-    <row r="71" spans="6:7">
+    <row r="71" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F71"/>
       <c r="G71"/>
     </row>
-    <row r="72" spans="6:7">
+    <row r="72" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F72"/>
       <c r="G72"/>
     </row>
-    <row r="73" spans="6:7">
+    <row r="73" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F73"/>
       <c r="G73"/>
     </row>
-    <row r="74" spans="6:7">
+    <row r="74" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F74"/>
       <c r="G74"/>
     </row>
-    <row r="75" spans="6:7">
+    <row r="75" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F75"/>
       <c r="G75"/>
     </row>
-    <row r="76" spans="6:7">
+    <row r="76" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F76"/>
       <c r="G76"/>
     </row>
-    <row r="77" spans="6:7">
+    <row r="77" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F77"/>
       <c r="G77"/>
     </row>
-    <row r="85" spans="6:7">
-      <c r="F85" s="45"/>
-      <c r="G85" s="45"/>
-    </row>
-    <row r="86" spans="6:7">
-      <c r="F86" s="45"/>
-      <c r="G86" s="45"/>
-    </row>
-    <row r="87" spans="6:7">
-      <c r="F87" s="45"/>
-      <c r="G87" s="45"/>
-    </row>
-    <row r="88" spans="6:7">
-      <c r="F88" s="45"/>
-      <c r="G88" s="45"/>
-    </row>
-    <row r="89" spans="6:7">
-      <c r="F89" s="45"/>
-      <c r="G89" s="45"/>
-    </row>
-    <row r="90" spans="6:7">
-      <c r="F90" s="45"/>
-      <c r="G90" s="45"/>
-    </row>
-    <row r="91" spans="6:7">
-      <c r="F91" s="45"/>
-      <c r="G91" s="45"/>
-    </row>
-    <row r="92" spans="6:7">
-      <c r="F92" s="45"/>
-      <c r="G92" s="45"/>
-    </row>
-    <row r="93" spans="6:7">
-      <c r="F93" s="45"/>
-      <c r="G93" s="45"/>
-    </row>
-    <row r="94" spans="6:7">
-      <c r="F94" s="45"/>
-      <c r="G94" s="45"/>
-    </row>
-    <row r="95" spans="6:7">
-      <c r="F95" s="45"/>
-      <c r="G95" s="45"/>
-    </row>
-    <row r="96" spans="6:7">
-      <c r="F96" s="45"/>
-      <c r="G96" s="45"/>
-    </row>
-    <row r="97" spans="6:7">
-      <c r="F97" s="45"/>
-      <c r="G97" s="45"/>
-    </row>
-    <row r="98" spans="6:7">
-      <c r="F98" s="45"/>
-      <c r="G98" s="45"/>
-    </row>
-    <row r="99" spans="6:7">
-      <c r="F99" s="45"/>
-      <c r="G99" s="45"/>
-    </row>
-    <row r="100" spans="6:7">
-      <c r="F100" s="45"/>
-      <c r="G100" s="45"/>
-    </row>
-    <row r="101" spans="6:7">
-      <c r="F101" s="45"/>
-      <c r="G101" s="45"/>
-    </row>
-    <row r="102" spans="6:7">
-      <c r="F102" s="45"/>
-      <c r="G102" s="45"/>
-    </row>
-    <row r="103" spans="6:7">
-      <c r="F103" s="45"/>
-      <c r="G103" s="45"/>
-    </row>
-    <row r="104" spans="6:7">
-      <c r="F104" s="45"/>
-      <c r="G104" s="45"/>
-    </row>
-    <row r="105" spans="6:7">
-      <c r="F105" s="45"/>
-      <c r="G105" s="45"/>
-    </row>
-    <row r="106" spans="6:7">
-      <c r="F106" s="45"/>
-      <c r="G106" s="45"/>
-    </row>
-    <row r="107" spans="6:7">
-      <c r="F107" s="45"/>
-      <c r="G107" s="45"/>
-    </row>
-    <row r="108" spans="6:7">
-      <c r="F108" s="45"/>
-      <c r="G108" s="45"/>
-    </row>
-    <row r="109" spans="6:7">
-      <c r="F109" s="45"/>
-      <c r="G109" s="45"/>
-    </row>
-    <row r="110" spans="6:7">
-      <c r="F110" s="45"/>
-      <c r="G110" s="45"/>
-    </row>
-    <row r="111" spans="6:7">
-      <c r="F111" s="45"/>
-      <c r="G111" s="45"/>
-    </row>
-    <row r="112" spans="6:7">
-      <c r="F112" s="45"/>
-      <c r="G112" s="45"/>
-    </row>
-    <row r="113" spans="6:7">
-      <c r="F113" s="45"/>
-      <c r="G113" s="45"/>
-    </row>
-    <row r="114" spans="6:7">
-      <c r="F114" s="45"/>
-      <c r="G114" s="45"/>
-    </row>
-    <row r="115" spans="6:7">
-      <c r="F115" s="45"/>
-      <c r="G115" s="45"/>
-    </row>
-    <row r="116" spans="6:7">
-      <c r="F116" s="45"/>
-      <c r="G116" s="45"/>
-    </row>
-    <row r="117" spans="6:7">
-      <c r="F117" s="45"/>
-      <c r="G117" s="45"/>
-    </row>
-    <row r="118" spans="6:7">
-      <c r="F118" s="45"/>
-      <c r="G118" s="45"/>
-    </row>
-    <row r="119" spans="6:7">
-      <c r="F119" s="45"/>
-      <c r="G119" s="45"/>
-    </row>
-    <row r="120" spans="6:7">
-      <c r="F120" s="45"/>
-      <c r="G120" s="45"/>
-    </row>
-    <row r="121" spans="6:7">
-      <c r="F121" s="45"/>
-      <c r="G121" s="45"/>
-    </row>
-    <row r="122" spans="6:7">
+    <row r="85" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F85" s="44"/>
+      <c r="G85" s="44"/>
+    </row>
+    <row r="86" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F86" s="44"/>
+      <c r="G86" s="44"/>
+    </row>
+    <row r="87" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F87" s="44"/>
+      <c r="G87" s="44"/>
+    </row>
+    <row r="88" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F88" s="44"/>
+      <c r="G88" s="44"/>
+    </row>
+    <row r="89" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F89" s="44"/>
+      <c r="G89" s="44"/>
+    </row>
+    <row r="90" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F90" s="44"/>
+      <c r="G90" s="44"/>
+    </row>
+    <row r="91" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F91" s="44"/>
+      <c r="G91" s="44"/>
+    </row>
+    <row r="92" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F92" s="44"/>
+      <c r="G92" s="44"/>
+    </row>
+    <row r="93" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F93" s="44"/>
+      <c r="G93" s="44"/>
+    </row>
+    <row r="94" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F94" s="44"/>
+      <c r="G94" s="44"/>
+    </row>
+    <row r="95" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F95" s="44"/>
+      <c r="G95" s="44"/>
+    </row>
+    <row r="96" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F96" s="44"/>
+      <c r="G96" s="44"/>
+    </row>
+    <row r="97" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F97" s="44"/>
+      <c r="G97" s="44"/>
+    </row>
+    <row r="98" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F98" s="44"/>
+      <c r="G98" s="44"/>
+    </row>
+    <row r="99" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F99" s="44"/>
+      <c r="G99" s="44"/>
+    </row>
+    <row r="100" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F100" s="44"/>
+      <c r="G100" s="44"/>
+    </row>
+    <row r="101" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F101" s="44"/>
+      <c r="G101" s="44"/>
+    </row>
+    <row r="102" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F102" s="44"/>
+      <c r="G102" s="44"/>
+    </row>
+    <row r="103" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F103" s="44"/>
+      <c r="G103" s="44"/>
+    </row>
+    <row r="104" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F104" s="44"/>
+      <c r="G104" s="44"/>
+    </row>
+    <row r="105" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F105" s="44"/>
+      <c r="G105" s="44"/>
+    </row>
+    <row r="106" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F106" s="44"/>
+      <c r="G106" s="44"/>
+    </row>
+    <row r="107" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F107" s="44"/>
+      <c r="G107" s="44"/>
+    </row>
+    <row r="108" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F108" s="44"/>
+      <c r="G108" s="44"/>
+    </row>
+    <row r="109" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F109" s="44"/>
+      <c r="G109" s="44"/>
+    </row>
+    <row r="110" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F110" s="44"/>
+      <c r="G110" s="44"/>
+    </row>
+    <row r="111" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F111" s="44"/>
+      <c r="G111" s="44"/>
+    </row>
+    <row r="112" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F112" s="44"/>
+      <c r="G112" s="44"/>
+    </row>
+    <row r="113" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F113" s="44"/>
+      <c r="G113" s="44"/>
+    </row>
+    <row r="114" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F114" s="44"/>
+      <c r="G114" s="44"/>
+    </row>
+    <row r="115" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F115" s="44"/>
+      <c r="G115" s="44"/>
+    </row>
+    <row r="116" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F116" s="44"/>
+      <c r="G116" s="44"/>
+    </row>
+    <row r="117" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F117" s="44"/>
+      <c r="G117" s="44"/>
+    </row>
+    <row r="118" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F118" s="44"/>
+      <c r="G118" s="44"/>
+    </row>
+    <row r="119" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F119" s="44"/>
+      <c r="G119" s="44"/>
+    </row>
+    <row r="120" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F120" s="44"/>
+      <c r="G120" s="44"/>
+    </row>
+    <row r="121" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F121" s="44"/>
+      <c r="G121" s="44"/>
+    </row>
+    <row r="122" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F122"/>
       <c r="G122"/>
     </row>
-    <row r="123" spans="6:7">
+    <row r="123" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F123"/>
       <c r="G123"/>
     </row>
-    <row r="124" spans="6:7">
+    <row r="124" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F124"/>
       <c r="G124"/>
     </row>
-    <row r="125" spans="6:7">
+    <row r="125" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F125"/>
       <c r="G125"/>
     </row>
-    <row r="126" spans="6:7">
+    <row r="126" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F126"/>
       <c r="G126"/>
     </row>
-    <row r="127" spans="6:7">
+    <row r="127" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F127"/>
       <c r="G127"/>
     </row>
-    <row r="128" spans="6:7">
+    <row r="128" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F128"/>
       <c r="G128"/>
     </row>
-    <row r="129" spans="6:7">
+    <row r="129" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F129"/>
       <c r="G129"/>
     </row>
-    <row r="130" spans="6:7">
+    <row r="130" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F130"/>
       <c r="G130"/>
     </row>
-    <row r="131" spans="6:7">
+    <row r="131" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F131"/>
       <c r="G131"/>
     </row>
-    <row r="132" spans="6:7">
+    <row r="132" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F132"/>
       <c r="G132"/>
     </row>
-    <row r="133" spans="6:7">
+    <row r="133" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F133"/>
       <c r="G133"/>
     </row>
-    <row r="134" spans="6:7">
+    <row r="134" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F134"/>
       <c r="G134"/>
     </row>
-    <row r="135" spans="6:7">
+    <row r="135" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F135"/>
       <c r="G135"/>
     </row>
-    <row r="136" spans="6:7">
+    <row r="136" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F136"/>
       <c r="G136"/>
     </row>
-    <row r="137" spans="6:7">
+    <row r="137" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F137"/>
       <c r="G137"/>
     </row>
-    <row r="138" spans="6:7">
+    <row r="138" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F138"/>
       <c r="G138"/>
     </row>
-    <row r="139" spans="6:7">
+    <row r="139" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F139"/>
       <c r="G139"/>
     </row>
-    <row r="140" spans="6:7">
+    <row r="140" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F140"/>
       <c r="G140"/>
     </row>
-    <row r="141" spans="6:7">
+    <row r="141" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F141"/>
       <c r="G141"/>
     </row>
-    <row r="142" spans="6:7">
+    <row r="142" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F142"/>
       <c r="G142"/>
     </row>
-    <row r="143" spans="6:7">
+    <row r="143" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F143"/>
       <c r="G143"/>
     </row>
-    <row r="144" spans="6:7">
+    <row r="144" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F144"/>
       <c r="G144"/>
     </row>
-    <row r="145" spans="6:7">
+    <row r="145" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F145"/>
       <c r="G145"/>
     </row>
-    <row r="146" spans="6:7">
+    <row r="146" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F146"/>
       <c r="G146"/>
     </row>
-    <row r="147" spans="6:7">
+    <row r="147" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F147"/>
       <c r="G147"/>
     </row>
-    <row r="148" spans="6:7">
+    <row r="148" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F148"/>
       <c r="G148"/>
     </row>
-    <row r="149" spans="6:7">
+    <row r="149" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F149"/>
       <c r="G149"/>
     </row>
-    <row r="150" spans="6:7">
+    <row r="150" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F150"/>
       <c r="G150"/>
     </row>
-    <row r="151" spans="6:7">
+    <row r="151" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F151"/>
       <c r="G151"/>
     </row>
-    <row r="152" spans="6:7">
+    <row r="152" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F152"/>
       <c r="G152"/>
     </row>
-    <row r="153" spans="6:7">
+    <row r="153" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F153"/>
       <c r="G153"/>
     </row>
-    <row r="154" spans="6:7">
+    <row r="154" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F154"/>
       <c r="G154"/>
     </row>
-    <row r="155" spans="6:7">
+    <row r="155" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F155"/>
       <c r="G155"/>
     </row>
-    <row r="156" spans="6:7">
+    <row r="156" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F156"/>
       <c r="G156"/>
     </row>
-    <row r="157" spans="6:7">
+    <row r="157" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F157"/>
       <c r="G157"/>
     </row>
-    <row r="158" spans="6:7">
+    <row r="158" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F158"/>
       <c r="G158"/>
     </row>
-    <row r="159" spans="6:7">
+    <row r="159" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F159"/>
       <c r="G159"/>
     </row>
-    <row r="160" spans="6:7">
+    <row r="160" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F160"/>
       <c r="G160"/>
     </row>
-    <row r="161" spans="6:7">
+    <row r="161" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F161"/>
       <c r="G161"/>
     </row>
-    <row r="162" spans="6:7">
+    <row r="162" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F162"/>
       <c r="G162"/>
     </row>
-    <row r="163" spans="6:7">
+    <row r="163" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F163"/>
       <c r="G163"/>
     </row>
-    <row r="164" spans="6:7">
+    <row r="164" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F164"/>
       <c r="G164"/>
     </row>
-    <row r="165" spans="6:7">
+    <row r="165" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F165"/>
       <c r="G165"/>
     </row>
-    <row r="166" spans="6:7">
+    <row r="166" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F166"/>
       <c r="G166"/>
     </row>
-    <row r="167" spans="6:7">
+    <row r="167" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F167"/>
       <c r="G167"/>
     </row>
-    <row r="168" spans="6:7">
+    <row r="168" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F168"/>
       <c r="G168"/>
     </row>
-    <row r="169" spans="6:7">
+    <row r="169" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F169"/>
       <c r="G169"/>
     </row>
-    <row r="170" spans="6:7">
+    <row r="170" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F170"/>
       <c r="G170"/>
     </row>
-    <row r="171" spans="6:7">
+    <row r="171" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F171"/>
       <c r="G171"/>
     </row>
-    <row r="172" spans="6:7">
+    <row r="172" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F172"/>
       <c r="G172"/>
     </row>
-    <row r="173" spans="6:7">
+    <row r="173" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F173"/>
       <c r="G173"/>
     </row>
-    <row r="174" spans="6:7">
+    <row r="174" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F174"/>
       <c r="G174"/>
     </row>
-    <row r="175" spans="6:7">
+    <row r="175" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F175"/>
       <c r="G175"/>
     </row>
-    <row r="176" spans="6:7">
+    <row r="176" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F176"/>
       <c r="G176"/>
     </row>
-    <row r="177" spans="6:7">
+    <row r="177" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F177"/>
       <c r="G177"/>
     </row>
-    <row r="178" spans="6:7">
+    <row r="178" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F178"/>
       <c r="G178"/>
     </row>
-    <row r="179" spans="6:7">
+    <row r="179" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F179"/>
       <c r="G179"/>
     </row>
-    <row r="180" spans="6:7">
+    <row r="180" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F180"/>
       <c r="G180"/>
     </row>
-    <row r="181" spans="6:7">
+    <row r="181" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F181"/>
       <c r="G181"/>
     </row>
-    <row r="182" spans="6:7">
+    <row r="182" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F182"/>
       <c r="G182"/>
     </row>
-    <row r="183" spans="6:7">
+    <row r="183" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F183"/>
       <c r="G183"/>
     </row>
-    <row r="184" spans="6:7">
+    <row r="184" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F184"/>
       <c r="G184"/>
     </row>
-    <row r="185" spans="6:7">
+    <row r="185" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F185"/>
       <c r="G185"/>
     </row>
-    <row r="186" spans="6:7">
+    <row r="186" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F186"/>
       <c r="G186"/>
     </row>
-    <row r="187" spans="6:7">
+    <row r="187" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F187"/>
       <c r="G187"/>
     </row>
-    <row r="188" spans="6:7">
+    <row r="188" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F188"/>
       <c r="G188"/>
     </row>
-    <row r="189" spans="6:7">
+    <row r="189" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F189"/>
       <c r="G189"/>
     </row>
-    <row r="190" spans="6:7">
+    <row r="190" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F190"/>
       <c r="G190"/>
     </row>
-    <row r="191" spans="6:7">
+    <row r="191" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F191"/>
       <c r="G191"/>
     </row>
-    <row r="192" spans="6:7">
+    <row r="192" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F192"/>
       <c r="G192"/>
     </row>
-    <row r="193" spans="6:7">
+    <row r="193" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F193"/>
       <c r="G193"/>
     </row>
-    <row r="194" spans="6:7">
+    <row r="194" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F194"/>
       <c r="G194"/>
     </row>
-    <row r="195" spans="6:7">
+    <row r="195" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F195"/>
       <c r="G195"/>
     </row>
-    <row r="196" spans="6:7">
+    <row r="196" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F196"/>
       <c r="G196"/>
     </row>
-    <row r="197" spans="6:7">
+    <row r="197" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F197"/>
       <c r="G197"/>
     </row>
-    <row r="198" spans="6:7">
+    <row r="198" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F198"/>
       <c r="G198"/>
     </row>
-    <row r="199" spans="6:7">
+    <row r="199" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F199"/>
       <c r="G199"/>
     </row>
-    <row r="200" spans="6:7">
+    <row r="200" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F200"/>
       <c r="G200"/>
     </row>
-    <row r="201" spans="6:7">
+    <row r="201" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F201"/>
       <c r="G201"/>
     </row>
-    <row r="202" spans="6:7">
+    <row r="202" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F202"/>
       <c r="G202"/>
     </row>
-    <row r="203" spans="6:7">
+    <row r="203" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F203"/>
       <c r="G203"/>
     </row>
-    <row r="204" spans="6:7">
+    <row r="204" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F204"/>
       <c r="G204"/>
     </row>
-    <row r="205" spans="6:7">
+    <row r="205" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F205"/>
       <c r="G205"/>
     </row>
-    <row r="206" spans="6:7">
+    <row r="206" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F206"/>
       <c r="G206"/>
     </row>
-    <row r="207" spans="6:7">
+    <row r="207" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F207"/>
       <c r="G207"/>
     </row>
-    <row r="208" spans="6:7">
+    <row r="208" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F208"/>
       <c r="G208"/>
     </row>
-    <row r="209" spans="6:7">
+    <row r="209" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F209"/>
       <c r="G209"/>
     </row>
-    <row r="210" spans="6:7">
+    <row r="210" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F210"/>
       <c r="G210"/>
     </row>
-    <row r="211" spans="6:7">
+    <row r="211" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F211"/>
       <c r="G211"/>
     </row>
-    <row r="212" spans="6:7">
+    <row r="212" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F212"/>
       <c r="G212"/>
     </row>
-    <row r="213" spans="6:7">
+    <row r="213" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F213"/>
       <c r="G213"/>
     </row>
-    <row r="214" spans="6:7">
+    <row r="214" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F214"/>
       <c r="G214"/>
     </row>
-    <row r="215" spans="6:7">
+    <row r="215" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F215"/>
       <c r="G215"/>
     </row>
-    <row r="216" spans="6:7">
+    <row r="216" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F216"/>
       <c r="G216"/>
     </row>
-    <row r="217" spans="6:7">
+    <row r="217" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F217"/>
       <c r="G217"/>
     </row>
-    <row r="218" spans="6:7">
+    <row r="218" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F218"/>
       <c r="G218"/>
     </row>
-    <row r="219" spans="6:7">
+    <row r="219" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F219"/>
       <c r="G219"/>
     </row>
-    <row r="220" spans="6:7">
+    <row r="220" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F220"/>
       <c r="G220"/>
     </row>
@@ -3860,204 +3904,205 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E3D808-0A96-49B8-9476-3F0C73FE1CDA}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.9453125" customWidth="1"/>
-    <col min="2" max="2" width="30.3125" customWidth="1"/>
-    <col min="3" max="3" width="24.3671875" customWidth="1"/>
-    <col min="5" max="5" width="19.15625" customWidth="1"/>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" customWidth="1"/>
+    <col min="3" max="3" width="24.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="43" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="42" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="43" t="s">
+      <c r="C1" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="E1" s="43" t="s">
+      <c r="E1" s="42" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="44" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="43" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="43" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="44" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="D3" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="44" t="s">
+      <c r="E3" s="43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="44" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="D4" s="44" t="s">
+      <c r="D4" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E4" s="44" t="s">
+      <c r="E4" s="43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="44" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D5" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E5" s="44" t="s">
+      <c r="E5" s="43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="44" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="D6" s="44" t="s">
+      <c r="D6" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="44" t="s">
+      <c r="E6" s="43" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="44" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="43" t="s">
         <v>143</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D7" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="E7" s="44" t="s">
+      <c r="E7" s="43" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="44" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="43" t="s">
         <v>144</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="43" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="43" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D8" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="43" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="44" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="43" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="E9" s="43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="44" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="43" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="44" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="43" t="s">
         <v>152</v>
       </c>
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="43" t="s">
         <v>153</v>
       </c>
-      <c r="C11" s="44" t="s">
+      <c r="C11" s="43" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="44" t="s">
+      <c r="D11" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="E11" s="44" t="s">
+      <c r="E11" s="43" t="s">
         <v>156</v>
       </c>
     </row>

</xml_diff>